<commit_message>
Close measure approval gate gaps
</commit_message>
<xml_diff>
--- a/outputs/qbc_ig_mapping/QBC_FHIR_Mapping_TaskSpec_v1.0-preview.1.xlsx
+++ b/outputs/qbc_ig_mapping/QBC_FHIR_Mapping_TaskSpec_v1.0-preview.1.xlsx
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Field_Mapping_115'!$A$1:$U$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Architecture'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Data_Flow'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Data_Flow'!$A$1:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Formal_Mapping_115'!$A$1:$AD$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Approval_Register'!$A$1:$M$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Extension_Candidates'!$A$1:$H$9</definedName>
@@ -285,8 +285,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QBCDataFlow" displayName="QBCDataFlow" ref="A1:F6" headerRowCount="1">
-  <autoFilter ref="A1:F6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QBCDataFlow" displayName="QBCDataFlow" ref="A1:F7" headerRowCount="1">
+  <autoFilter ref="A1:F7"/>
   <tableColumns count="6">
     <tableColumn id="1" name="State"/>
     <tableColumn id="2" name="Input"/>
@@ -802,7 +802,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>目前：癌症診療計畫書 → QBC Task。目標：原始報告／系統 → BreastCancer canonical facts → 計畫書或直接 QBC／其他 Task。</t>
+          <t>唯一目標：原始報告／系統 → BreastCancer common FHIR facts → 平行的 Care Plan／QBC／其他 Task。現有診療計畫 JSON 只作 secondary source alignment check。</t>
         </is>
       </c>
       <c r="C7" s="2" t="n"/>
@@ -10717,7 +10717,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>102</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
@@ -10808,7 +10808,7 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>103</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
@@ -10899,7 +10899,7 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>104</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
@@ -10994,7 +10994,7 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>105</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
@@ -11089,7 +11089,7 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>106</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
@@ -11184,7 +11184,7 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>107</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
@@ -11279,7 +11279,7 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>108</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
@@ -11370,7 +11370,7 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>109</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
@@ -11461,7 +11461,7 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>110</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
@@ -11552,7 +11552,7 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>111</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
@@ -11647,7 +11647,7 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>112</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
@@ -11742,7 +11742,7 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>113</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
@@ -11833,7 +11833,7 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>114</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
@@ -11920,7 +11920,7 @@
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>115</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
@@ -12184,22 +12184,22 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Derived document/collaboration layer</t>
+          <t>Parallel task/document projections</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>clinical workflow</t>
+          <t>task-specific workflow</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Cancer diagnosis/treatment plan, treatment plan and MDT record</t>
+          <t>Cancer care plan, QBC, treatment plan and MDT record</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>generated from canonical facts; may be bridge input during migration</t>
+          <t>independently generated from common FHIR facts; no task-to-task production dependency</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -12226,7 +12226,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>reads canonical facts or current plan bridge input</t>
+          <t>reads common FHIR facts; secondary-source adapter is migration/check only</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -12250,7 +12250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12296,32 +12296,32 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Current bridge</t>
+          <t>Current secondary source</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書</t>
+          <t>癌症診療計畫書 JSON</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>document extraction + QBC review</t>
+          <t>independent Care Plan/QBC adapters + alignment check</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>partial; gradually normalize to BreastCancer facts</t>
+          <t>partial; gradually normalize to BreastCancer common FHIR facts</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>QBC FHIR Bundle → QBC XML</t>
+          <t>separate Care Plan and QBC check Bundles</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>plan is derived input, not original evidence</t>
+          <t>check only; neither task output is the other task input</t>
         </is>
       </c>
     </row>
@@ -12333,22 +12333,22 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書</t>
+          <t>癌症診療計畫書 JSON</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>bridge adapter + provenance + reconciliation</t>
+          <t>secondary-source adapter + provenance + reconciliation</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>BreastCancer canonical facts</t>
+          <t>BreastCancer common FHIR facts</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>QBC and regenerated treatment-plan document</t>
+          <t>parallel task projections</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -12360,7 +12360,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Target A</t>
+          <t>Target common layer</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -12370,17 +12370,17 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>source-specific mapping</t>
+          <t>source-specific mapping + provenance</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>BreastCancer canonical facts</t>
+          <t>BreastCancer common FHIR facts</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>generate cancer diagnosis/treatment plan</t>
+          <t>task-neutral fact store or exchange Bundle</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -12392,69 +12392,101 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Target B</t>
+          <t>Target Care Plan task</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>pathology/laboratory/ultrasound/treatment sources</t>
+          <t>BreastCancer common FHIR facts</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>source-specific mapping</t>
+          <t>Care Plan-specific projection</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>BreastCancer canonical facts</t>
+          <t>read-only common layer</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>direct QBC projection</t>
+          <t>Cancer Care Plan Bundle</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>same rules/version as plan-first pathway</t>
+          <t>parallel task; never feeds QBC production input</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Target C</t>
+          <t>Target QBC task</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>BreastCancer canonical facts</t>
+          <t>BreastCancer common FHIR facts + QBC-only fields</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
+          <t>QBC-specific projection</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>read-only common layer</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>QBC Bundle → QBC XML</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>parallel task; alignment with Care Plan is check-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Target other tasks</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>BreastCancer common FHIR facts</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
           <t>task-specific projection</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>single reusable fact store</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>read-only common layer</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>drug prior authorization / registry / treatment plan / MDT</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>task output never overwrites source facts silently</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F6"/>
+  <autoFilter ref="A1:F7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -14714,7 +14746,7 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
@@ -14866,7 +14898,7 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
@@ -15010,7 +15042,7 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
@@ -15162,7 +15194,7 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
@@ -15306,7 +15338,7 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
@@ -15458,7 +15490,7 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
@@ -15610,7 +15642,7 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
@@ -15762,7 +15794,7 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
@@ -15914,7 +15946,7 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
@@ -16066,7 +16098,7 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
@@ -16218,7 +16250,7 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
@@ -16362,7 +16394,7 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
@@ -16506,7 +16538,7 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
@@ -16650,7 +16682,7 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
@@ -16802,7 +16834,7 @@
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J30" s="6" t="inlineStr">
@@ -16954,7 +16986,7 @@
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J31" s="6" t="inlineStr">
@@ -17106,7 +17138,7 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr">
@@ -17258,7 +17290,7 @@
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J33" s="6" t="inlineStr">
@@ -17410,7 +17442,7 @@
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
@@ -17562,7 +17594,7 @@
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
@@ -17714,7 +17746,7 @@
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J36" s="6" t="inlineStr">
@@ -17866,7 +17898,7 @@
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
@@ -18018,7 +18050,7 @@
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
@@ -18170,7 +18202,7 @@
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
@@ -18314,7 +18346,7 @@
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr">
@@ -18466,7 +18498,7 @@
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J41" s="6" t="inlineStr">
@@ -18610,7 +18642,7 @@
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J42" s="6" t="inlineStr">
@@ -18754,7 +18786,7 @@
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J43" s="6" t="inlineStr">
@@ -18898,7 +18930,7 @@
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J44" s="6" t="inlineStr">
@@ -19042,7 +19074,7 @@
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J45" s="6" t="inlineStr">
@@ -19194,7 +19226,7 @@
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J46" s="6" t="inlineStr">
@@ -19338,7 +19370,7 @@
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J47" s="6" t="inlineStr">
@@ -19490,7 +19522,7 @@
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J48" s="6" t="inlineStr">
@@ -19642,7 +19674,7 @@
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J49" s="6" t="inlineStr">
@@ -19794,7 +19826,7 @@
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J50" s="6" t="inlineStr">
@@ -19946,7 +19978,7 @@
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J51" s="6" t="inlineStr">
@@ -20098,7 +20130,7 @@
       </c>
       <c r="I52" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J52" s="6" t="inlineStr">
@@ -20250,7 +20282,7 @@
       </c>
       <c r="I53" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J53" s="6" t="inlineStr">
@@ -20402,7 +20434,7 @@
       </c>
       <c r="I54" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J54" s="6" t="inlineStr">
@@ -20546,7 +20578,7 @@
       </c>
       <c r="I55" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J55" s="6" t="inlineStr">
@@ -20690,7 +20722,7 @@
       </c>
       <c r="I56" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J56" s="6" t="inlineStr">
@@ -20842,7 +20874,7 @@
       </c>
       <c r="I57" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J57" s="6" t="inlineStr">
@@ -20986,7 +21018,7 @@
       </c>
       <c r="I58" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J58" s="6" t="inlineStr">
@@ -21130,7 +21162,7 @@
       </c>
       <c r="I59" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J59" s="6" t="inlineStr">
@@ -21274,7 +21306,7 @@
       </c>
       <c r="I60" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J60" s="6" t="inlineStr">
@@ -21418,7 +21450,7 @@
       </c>
       <c r="I61" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J61" s="6" t="inlineStr">
@@ -21562,7 +21594,7 @@
       </c>
       <c r="I62" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J62" s="6" t="inlineStr">
@@ -21706,7 +21738,7 @@
       </c>
       <c r="I63" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J63" s="6" t="inlineStr">
@@ -21858,7 +21890,7 @@
       </c>
       <c r="I64" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J64" s="6" t="inlineStr">
@@ -22010,7 +22042,7 @@
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J65" s="6" t="inlineStr">
@@ -22162,7 +22194,7 @@
       </c>
       <c r="I66" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J66" s="6" t="inlineStr">
@@ -22314,7 +22346,7 @@
       </c>
       <c r="I67" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J67" s="6" t="inlineStr">
@@ -22466,7 +22498,7 @@
       </c>
       <c r="I68" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J68" s="6" t="inlineStr">
@@ -22618,7 +22650,7 @@
       </c>
       <c r="I69" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J69" s="6" t="inlineStr">
@@ -22770,7 +22802,7 @@
       </c>
       <c r="I70" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J70" s="6" t="inlineStr">
@@ -22922,7 +22954,7 @@
       </c>
       <c r="I71" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J71" s="6" t="inlineStr">
@@ -23074,7 +23106,7 @@
       </c>
       <c r="I72" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr">
@@ -23226,7 +23258,7 @@
       </c>
       <c r="I73" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J73" s="6" t="inlineStr">
@@ -23378,7 +23410,7 @@
       </c>
       <c r="I74" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J74" s="6" t="inlineStr">
@@ -23522,7 +23554,7 @@
       </c>
       <c r="I75" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr">
@@ -23674,7 +23706,7 @@
       </c>
       <c r="I76" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J76" s="6" t="inlineStr">
@@ -23826,7 +23858,7 @@
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr">
@@ -23978,7 +24010,7 @@
       </c>
       <c r="I78" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J78" s="6" t="inlineStr">
@@ -24130,7 +24162,7 @@
       </c>
       <c r="I79" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J79" s="6" t="inlineStr">
@@ -24282,7 +24314,7 @@
       </c>
       <c r="I80" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J80" s="6" t="inlineStr">
@@ -24434,7 +24466,7 @@
       </c>
       <c r="I81" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J81" s="6" t="inlineStr">
@@ -24586,7 +24618,7 @@
       </c>
       <c r="I82" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J82" s="6" t="inlineStr">
@@ -24738,7 +24770,7 @@
       </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J83" s="6" t="inlineStr">
@@ -24890,7 +24922,7 @@
       </c>
       <c r="I84" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J84" s="6" t="inlineStr">
@@ -25042,7 +25074,7 @@
       </c>
       <c r="I85" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J85" s="6" t="inlineStr">
@@ -25194,7 +25226,7 @@
       </c>
       <c r="I86" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J86" s="6" t="inlineStr">
@@ -25338,7 +25370,7 @@
       </c>
       <c r="I87" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J87" s="6" t="inlineStr">
@@ -25482,7 +25514,7 @@
       </c>
       <c r="I88" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J88" s="6" t="inlineStr">
@@ -25634,7 +25666,7 @@
       </c>
       <c r="I89" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J89" s="6" t="inlineStr">
@@ -25778,7 +25810,7 @@
       </c>
       <c r="I90" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J90" s="6" t="inlineStr">
@@ -25922,7 +25954,7 @@
       </c>
       <c r="I91" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J91" s="6" t="inlineStr">
@@ -26074,7 +26106,7 @@
       </c>
       <c r="I92" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J92" s="6" t="inlineStr">
@@ -26226,7 +26258,7 @@
       </c>
       <c r="I93" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J93" s="6" t="inlineStr">
@@ -26378,7 +26410,7 @@
       </c>
       <c r="I94" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J94" s="6" t="inlineStr">
@@ -26530,7 +26562,7 @@
       </c>
       <c r="I95" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J95" s="6" t="inlineStr">
@@ -26682,7 +26714,7 @@
       </c>
       <c r="I96" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J96" s="6" t="inlineStr">
@@ -26834,7 +26866,7 @@
       </c>
       <c r="I97" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J97" s="6" t="inlineStr">
@@ -26986,7 +27018,7 @@
       </c>
       <c r="I98" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J98" s="6" t="inlineStr">
@@ -27138,7 +27170,7 @@
       </c>
       <c r="I99" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J99" s="6" t="inlineStr">
@@ -27290,7 +27322,7 @@
       </c>
       <c r="I100" s="6" t="inlineStr">
         <is>
-          <t>癌症診療計畫書（目前 bridge input）</t>
+          <t>癌症診療計畫書 JSON（過渡期 secondary source；非 Care Plan Task 輸出）</t>
         </is>
       </c>
       <c r="J100" s="6" t="inlineStr">

</xml_diff>